<commit_message>
Correct showcase financial labels and sharpen evidence boundaries
Refresh real Nexus captures and synthetic inputs. Make the founder's product judgment explicit and describe orchestration without publishing private source contracts or verification results.

Co-Authored-By: GPT-6 <noreply@openai.com>
Agent-Role: builder
Agent-Run: main
</commit_message>
<xml_diff>
--- a/assets/demo/northstar-pilot-economics.xlsx
+++ b/assets/demo/northstar-pilot-economics.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot economics" sheetId="1" r:id="Rbbdacef21e48419b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilot economics" sheetId="1" r:id="R8159313f7e284036"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -448,7 +448,7 @@
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
       <x:c r="A12" s="13" t="str">
-        <x:v>Monthly contribution</x:v>
+        <x:v>Operating surplus</x:v>
       </x:c>
       <x:c r="B12" s="14" t="n">
         <x:f>B8-B10-B11</x:f>
@@ -464,7 +464,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="13" t="str">
-        <x:v>Contribution margin</x:v>
+        <x:v>Surplus margin</x:v>
       </x:c>
       <x:c r="B13" s="15" t="n">
         <x:f>B12/B8</x:f>

</xml_diff>